<commit_message>
Automatiza 22 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/PINTURA/LISTA PINTURA PG + ECO HIBRIDO LADO MENOR.xlsx
+++ b/PINTURA/LISTA PINTURA PG + ECO HIBRIDO LADO MENOR.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Plan1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -44,11 +44,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -327,13 +326,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="6"/>
+    <col width="42" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
@@ -392,7 +391,7 @@
       <c r="E2" t="n">
         <v>4000</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>001469</t>
         </is>
@@ -420,7 +419,7 @@
       <c r="E3" t="n">
         <v>4000</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>001470</t>
         </is>
@@ -448,7 +447,7 @@
       <c r="E4" t="n">
         <v>1000</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>001471</t>
         </is>
@@ -476,7 +475,7 @@
       <c r="E5" t="n">
         <v>1000</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>001472</t>
         </is>
@@ -504,7 +503,7 @@
       <c r="E6" t="n">
         <v>1000</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>001473</t>
         </is>
@@ -532,7 +531,7 @@
       <c r="E7" t="n">
         <v>1000</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>001474</t>
         </is>
@@ -560,7 +559,7 @@
       <c r="E8" t="n">
         <v>1000</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>001475</t>
         </is>
@@ -588,7 +587,7 @@
       <c r="E9" t="n">
         <v>1000</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>001476</t>
         </is>
@@ -602,23 +601,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Retorno da Pintura</t>
+          <t>Envio á Pintura</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BDJ ESQUERDA MENOR CORPO - RETORNO</t>
+          <t>CHAVE - ENVIO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>001477</t>
+        <v>1000</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>001489</t>
         </is>
       </c>
     </row>
@@ -630,23 +629,23 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Retorno da Pintura</t>
+          <t>Envio á Pintura</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BDJ DIREITA MAIOR CORPO - RETORNO</t>
+          <t>SUPORTE FIXAÇÃO - ENVIO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>001478</t>
+        <v>2000</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>001490</t>
         </is>
       </c>
     </row>
@@ -663,18 +662,18 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BDJ ESQUERDA MENOR BASE - RETORNO</t>
+          <t>BDJ ESQUERDA MENOR CORPO - RETORNO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>001479</t>
+        <v>4000</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>001477</t>
         </is>
       </c>
     </row>
@@ -691,18 +690,18 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BDJ DIREITA MAIOR BASE - RETORNO</t>
+          <t>BDJ DIREITA MAIOR CORPO - RETORNO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>001480</t>
+        <v>4000</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>001478</t>
         </is>
       </c>
     </row>
@@ -719,7 +718,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CORPO - RETORNO</t>
+          <t>BDJ ESQUERDA MENOR BASE - RETORNO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -728,9 +727,9 @@
       <c r="E14" t="n">
         <v>1000</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>001481</t>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>001479</t>
         </is>
       </c>
     </row>
@@ -747,7 +746,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TOLDO - RETORNO</t>
+          <t>BDJ DIREITA MAIOR BASE - RETORNO</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -756,9 +755,9 @@
       <c r="E15" t="n">
         <v>1000</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>001482</t>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>001480</t>
         </is>
       </c>
     </row>
@@ -775,7 +774,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FECHAMENTO MÓVEL - RETORNO</t>
+          <t>CORPO - RETORNO</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -784,9 +783,9 @@
       <c r="E16" t="n">
         <v>1000</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>001483</t>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>001481</t>
         </is>
       </c>
     </row>
@@ -803,18 +802,130 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>TOLDO - RETORNO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>001482</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PG + ECONOMIA HIBRIDO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Retorno da Pintura</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FECHAMENTO MÓVEL - RETORNO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>001483</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PG + ECONOMIA HIBRIDO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Retorno da Pintura</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>PARACHOQUE - RETORNO</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>001484</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PG + ECONOMIA HIBRIDO</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Retorno da Pintura</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CHAVE - RETORNO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>001491</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PG + ECONOMIA HIBRIDO</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Retorno da Pintura</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SUPORTE FIXAÇÃO - RETORNO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>001492</t>
         </is>
       </c>
     </row>

</xml_diff>